<commit_message>
database: museum guide, generic import, DeepL translation, removal of first names and obsolete scripts
</commit_message>
<xml_diff>
--- a/database/PP1-Collection_Database.xlsx
+++ b/database/PP1-Collection_Database.xlsx
@@ -9,12 +9,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Database" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="List of questions" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transcriptions" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="noms" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Type of object" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Type of object" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Database'!$A$2:$Q$118</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Type of object'!$A$2:$A$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Type of object'!$A$2:$A$28</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -15665,12 +15664,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:B14"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
     <col width="67.5546875" customWidth="1" style="1" min="2" max="2"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
         <is>
@@ -18086,631 +18086,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A86"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
-  <cols>
-    <col width="25" bestFit="1" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Alexandru</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Isabelle</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Emilien Dubuc</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Amel</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="43.2" customHeight="1">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>Godfried, Edmond, Pierre, Marie</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>Marc</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>Hermann</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>Arnold</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>Georges</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>Titus</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>Louis, Pierre</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>Albert</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="28.8" customHeight="1">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>Constant Devreese</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t>Harald, Bertrand</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>Henri</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Sophie, Félicité</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Nicolas</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Michel, Cécile</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Pierre</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Constant</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Dorothée, Joseph</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Armand</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Jean, Baptiste, Octave</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Eugénie, Sophie</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Marie-Thérèse</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Joseph</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Nicolas, Louis</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Arnould</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Louise</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Agathe</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Paul</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Claire</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Sophie, Benoit, Ghislain</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Louis</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Cesar</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Georges</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Gustave, Joseph, Jean</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>Nicolas</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>Joseph, Joachim, Anna, Marie</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>Désirée, Eloi</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>Guillaume</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>Antoine</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>Alexandrine, Françoise</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>Henri</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>Marie, Emilie, Françoise</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>Nicolas, Bernard</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>Benoit, Ghislain</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>Benoit, Ghislain</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>Jeanne, Françoise, Chantal</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>Sophie</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>Marie, Aldegonde</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Virginie, </t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>Lucie</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>Charles, Rose</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>Flore, Marc</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>Rosalie</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>Zoé, Hélène</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>Eugénie</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>Alexandrine, Sophie</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>Julie</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>Juliette</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>Geneviève</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>Adrien</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>Barthelemy, Joseph</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>Laurent</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>Benoit, Ghislain</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>Françoise</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>Joseph</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>François, Louis</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>Charlotte, Colette</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>Victoire</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>Marie, Joseph</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>Charles</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>Michiel, Eloi</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>Andreas, Gabrielle</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>Pauline</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>Louis</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>Joséphine</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>Adelaide</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>Charles</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>Joseph, Gabriel</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t>Elisabeth</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>Henri, Victor</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>Waudru</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t>Louis</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>Narcisse</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A2:A28"/>
+  <dimension ref="A1:A28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
     <col width="28.88671875" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>

</xml_diff>